<commit_message>
feat(import): flag copied and suspect rows in the b023 crop table (#289)
Both importers now warn, per crop, when a [Crop demand] row repeats an
earlier crop's 12 factors, or has a negative factor, a lone 0, a lone
spike or dip of more than 0.3 against both neighbours, or a factor above
1.0. The factors still import unchanged. The synthetic fixture gains a
copied row and a crop with slips, so the parity tests cover the text.
</commit_message>
<xml_diff>
--- a/scripts/wbt-import/fixtures/synthetic_b023.xlsx
+++ b/scripts/wbt-import/fixtures/synthetic_b023.xlsx
@@ -62,14 +62,14 @@
     <definedName name="zFarmSpec_CompositeDamMinPerc">'Farm spec'!$R$30:$R$39</definedName>
     <definedName name="zFarmSpec_DiversionToDam">'Farm spec'!$T$30:$T$39</definedName>
     <definedName name="zFarmSpec_PercIrrReturnFlow">'Farm spec'!$U$30:$U$39</definedName>
-    <definedName name="zCropDemand_CropNameLst">'Crop demand'!$D$30:$D$36</definedName>
-    <definedName name="zCropDemand_FactorsTbl">'Crop demand'!$E$30:$R$36</definedName>
-    <definedName name="zCropDemand_GrossTbl">'Crop demand'!$R$30:$AE$36</definedName>
+    <definedName name="zCropDemand_CropNameLst">'Crop demand'!$D$30:$D$37</definedName>
+    <definedName name="zCropDemand_FactorsTbl">'Crop demand'!$E$30:$R$37</definedName>
+    <definedName name="zCropDemand_GrossTbl">'Crop demand'!$R$30:$AE$37</definedName>
     <definedName name="rCropDemand_EffectiveRainfall">'Crop demand'!$F$23</definedName>
     <definedName name="rCropDemand_CalcPrecision">'Crop demand'!$F$12</definedName>
     <definedName name="zFarmDemand_FarmNameLst">'Farm demand'!$D$24:$D$35</definedName>
-    <definedName name="zFarmDemand_CropNameLst">'Farm demand'!$G$24:$N$24</definedName>
-    <definedName name="zFarmDemand_FarmCropAreaTotalLst">'Farm demand'!$O$24:$O$35</definedName>
+    <definedName name="zFarmDemand_CropNameLst">'Farm demand'!$G$24:$O$24</definedName>
+    <definedName name="zFarmDemand_FarmCropAreaTotalLst">'Farm demand'!$P$24:$P$35</definedName>
     <definedName name="zFarmDemand_GrossMth">'Farm demand'!$Q$24:$AB$35</definedName>
     <definedName name="zFarmDemand_GrossMthDays">'Farm demand'!$Q$19:$AB$19</definedName>
     <definedName name="zTransfers_HeaderDate">Transfers!$G$19</definedName>
@@ -47806,7 +47806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD36"/>
+  <dimension ref="A1:AD37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48476,7 +48476,7 @@
         <v>0.5</v>
       </c>
       <c r="H35" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>0.5</v>
@@ -48485,7 +48485,7 @@
         <v>0.5</v>
       </c>
       <c r="K35" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="L35" t="n">
         <v>0.5</v>
@@ -48512,7 +48512,7 @@
         <v>120</v>
       </c>
       <c r="U35" t="n">
-        <v>142.5</v>
+        <v>0</v>
       </c>
       <c r="V35" t="n">
         <v>150</v>
@@ -48521,7 +48521,7 @@
         <v>125</v>
       </c>
       <c r="X35" t="n">
-        <v>112.5</v>
+        <v>270</v>
       </c>
       <c r="Y35" t="n">
         <v>75</v>
@@ -48545,125 +48545,204 @@
     <row r="36">
       <c r="D36" t="inlineStr">
         <is>
+          <t>Pasture F</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="S36" t="n">
+        <v>133</v>
+      </c>
+      <c r="T36" t="n">
+        <v>180</v>
+      </c>
+      <c r="U36" t="n">
+        <v>228</v>
+      </c>
+      <c r="V36" t="n">
+        <v>240</v>
+      </c>
+      <c r="W36" t="n">
+        <v>200</v>
+      </c>
+      <c r="X36" t="n">
+        <v>180</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>57</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="AB36" t="n">
+        <v>35</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="D37" t="inlineStr">
+        <is>
           <t>-- do NOT delete this row !  Insert here</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="P37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr">
+      <c r="Q37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
+      <c r="S37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="T36" t="inlineStr">
+      <c r="T37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="U37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="V36" t="inlineStr">
+      <c r="V37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="W36" t="inlineStr">
+      <c r="W37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr">
+      <c r="X37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="Y36" t="inlineStr">
+      <c r="Y37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="Z36" t="inlineStr">
+      <c r="Z37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="AA36" t="inlineStr">
+      <c r="AA37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="AB36" t="inlineStr">
+      <c r="AB37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="AC36" t="inlineStr">
+      <c r="AC37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="AD36" t="inlineStr">
+      <c r="AD37" t="inlineStr">
         <is>
           <t>--</t>
         </is>
@@ -48849,15 +48928,20 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
+          <t>Pasture F</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
           <t>Hops X</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>|</t>
-        </is>
-      </c>
       <c r="O24" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -48960,12 +49044,15 @@
       <c r="M25" t="n">
         <v>0</v>
       </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>|</t>
-        </is>
-      </c>
-      <c r="O25" t="n">
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
         <v>200000</v>
       </c>
       <c r="Q25" t="n">
@@ -49039,12 +49126,15 @@
       <c r="M26" t="n">
         <v>0</v>
       </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>|</t>
-        </is>
-      </c>
-      <c r="O26" t="n">
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
         <v>210000</v>
       </c>
       <c r="Q26" t="n">
@@ -49121,12 +49211,15 @@
       <c r="M27" t="n">
         <v>0</v>
       </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>|</t>
-        </is>
-      </c>
-      <c r="O27" t="n">
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
         <v>0</v>
       </c>
       <c r="Q27" t="n">
@@ -49201,14 +49294,17 @@
         <v>0</v>
       </c>
       <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
         <v>25000</v>
       </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>|</t>
-        </is>
-      </c>
-      <c r="O29" t="n">
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
         <v>275000</v>
       </c>
       <c r="Q29" t="n">
@@ -49285,12 +49381,15 @@
       <c r="M30" t="n">
         <v>0</v>
       </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>|</t>
-        </is>
-      </c>
-      <c r="O30" t="n">
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
         <v>90000</v>
       </c>
       <c r="Q30" t="n">
@@ -49367,12 +49466,15 @@
       <c r="M31" t="n">
         <v>0</v>
       </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>|</t>
-        </is>
-      </c>
-      <c r="O31" t="n">
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
         <v>75000</v>
       </c>
       <c r="Q31" t="n">
@@ -49449,12 +49551,15 @@
       <c r="M32" t="n">
         <v>0</v>
       </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>|</t>
-        </is>
-      </c>
-      <c r="O32" t="n">
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
         <v>70000</v>
       </c>
       <c r="Q32" t="n">
@@ -49531,12 +49636,15 @@
       <c r="M33" t="n">
         <v>0</v>
       </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>|</t>
-        </is>
-      </c>
-      <c r="O33" t="n">
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
         <v>40000</v>
       </c>
       <c r="Q33" t="n">
@@ -49613,12 +49721,15 @@
       <c r="M34" t="n">
         <v>0</v>
       </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>|</t>
-        </is>
-      </c>
-      <c r="O34" t="n">
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
         <v>50000</v>
       </c>
       <c r="Q34" t="n">
@@ -49715,6 +49826,11 @@
         </is>
       </c>
       <c r="O35" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
         <is>
           <t>--</t>
         </is>

</xml_diff>

<commit_message>
fix(import): make workbook names one line in both importers (#385)
clean() in extract_project.py and the browser importer now turns every run
of whitespace and C0, DEL and C1 control characters into one space, so a
multi-line or pasted cell can't give a node or crop a name the model schema
is about to refuse. The synthetic b023 fixture gains a cell line break
(Golf Farm in [Network]) and a U+009F in a crop name; the committed project
JSON is unchanged, which is the parity check that both sides clean them.
</commit_message>
<xml_diff>
--- a/scripts/wbt-import/fixtures/synthetic_b023.xlsx
+++ b/scripts/wbt-import/fixtures/synthetic_b023.xlsx
@@ -46793,7 +46793,8 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Golf Farm</t>
+          <t>Golf
+Farm</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -48387,7 +48388,7 @@
     <row r="34">
       <c r="D34" t="inlineStr">
         <is>
-          <t>Vines D</t>
+          <t>VinesD</t>
         </is>
       </c>
       <c r="F34" t="n">

</xml_diff>